<commit_message>
Cambio el formato de numero a texto detro de la columna de los Id's para solucionar el error, no mostrar consulta por diferente formato
</commit_message>
<xml_diff>
--- a/backend/datos.xlsx
+++ b/backend/datos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon cifuentes\Desktop\repositorio-david\metodologias-software\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\Repositorio\metodologias-software\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69F2624-D395-4C65-87C4-80A95C7ED65C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBB792E-1561-4C1E-8ED9-B3BA6D2BD849}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="productos" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>id</t>
   </si>
@@ -67,16 +70,52 @@
   </si>
   <si>
     <t>cebolla</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>10</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -102,9 +141,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -386,13 +426,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="18.109375" customWidth="1"/>
-    <col min="3" max="3" width="16.21875" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" customWidth="1"/>
+    <col min="3" max="3" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -406,9 +446,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2">
-        <v>1</v>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
@@ -420,9 +460,9 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3">
-        <v>2</v>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -434,9 +474,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4">
-        <v>3</v>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>16</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -448,9 +488,9 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5">
-        <v>4</v>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>7</v>
@@ -462,9 +502,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6">
-        <v>5</v>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>18</v>
       </c>
       <c r="B6" t="s">
         <v>8</v>
@@ -476,9 +516,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7">
-        <v>6</v>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="B7" t="s">
         <v>9</v>
@@ -490,9 +530,9 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8">
-        <v>7</v>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="B8" t="s">
         <v>10</v>
@@ -504,9 +544,9 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9">
-        <v>8</v>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="B9" t="s">
         <v>11</v>
@@ -518,9 +558,9 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10">
-        <v>9</v>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>22</v>
       </c>
       <c r="B10" t="s">
         <v>12</v>
@@ -532,9 +572,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11">
-        <v>10</v>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="B11" t="s">
         <v>13</v>
@@ -547,6 +587,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>